<commit_message>
fix(import): indirim, telefon ve not disa/ice aktarma turunda korunur
Sablon sutunlarina Oda Indirimi, Telefon ve Not eklendi (tek kaynak
SABLON_SUTUNLARI: ornek sablon, disa aktarma, esleme). Indirim oda
gelirini asamaz. Geri yuklenen rezervasyonun cirosu artik indirim kadar
sismez (L-39). Ornek sablonlar ureticiyle yeniden uretildi.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablonlar/lexbnb-rezervasyon-sablonu.xlsx
+++ b/sablonlar/lexbnb-rezervasyon-sablonu.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:M3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,6 +431,15 @@
       <c r="J1" t="str">
         <v>Durum</v>
       </c>
+      <c r="K1" t="str">
+        <v>Oda İndirimi (TL)</v>
+      </c>
+      <c r="L1" t="str">
+        <v>Telefon</v>
+      </c>
+      <c r="M1" t="str">
+        <v>Not</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -463,6 +472,15 @@
       <c r="J2" t="str">
         <v>CONFIRMED</v>
       </c>
+      <c r="K2" t="str">
+        <v>2500</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v>Örnek not</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -495,17 +513,26 @@
       <c r="J3" t="str">
         <v>CONFIRMED</v>
       </c>
+      <c r="K3" t="str">
+        <v>0</v>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A19"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -584,17 +611,27 @@
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v/>
+        <v>8) "Oda İndirimi" yalnız oda gelirinden düşer; temizlik ücretini etkilemez.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
+        <v xml:space="preserve">   "Telefon" ve "Not" isteğe bağlıdır.</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
         <v>Durum değerleri: CONFIRMED, CHECKED_IN, CHECKED_OUT, CANCELLED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ledger): cleaning column says it is the fee taken from the guest [G9-M23]
The booking ledger's cleaning column is income (cleaning_fee); users
read 0 as missing cleaning cost. Header is now 'Misafirden Temizlik
Ucreti (TL)'; the old header stays an alias so earlier files still
import. Template notes say the staff cost is not in this file.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sablonlar/lexbnb-rezervasyon-sablonu.xlsx
+++ b/sablonlar/lexbnb-rezervasyon-sablonu.xlsx
@@ -423,7 +423,7 @@
         <v>OTA Komisyonu (TL)</v>
       </c>
       <c r="H1" t="str">
-        <v>Temizlik Ücreti (TL)</v>
+        <v>Misafirden Temizlik Ücreti (TL)</v>
       </c>
       <c r="I1" t="str">
         <v>Kişi Sayısı</v>
@@ -532,7 +532,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A19"/>
+  <dimension ref="A1:A20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -586,52 +586,57 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>4) Brüt tutar temizlik ücretini İÇERİR; ayrıca "Temizlik Ücreti" sütununa</v>
+        <v>4) "Misafirden Temizlik Ücreti": misafirden ALINAN temizlik ücretidir (gelir);</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v xml:space="preserve">   yazdığınız kısım gelir olarak ayrı raporlanır.</v>
+        <v xml:space="preserve">   brüt tutarın içindedir ve ayrı raporlanır. Personele ödenen temizlik</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>5) Gece sayısı tarihlerden hesaplanır, ayrı sütun gerekmez.</v>
+        <v xml:space="preserve">   MALİYETİ bu dosyada yoktur; temizlik görevinden gider olarak yazılır.</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>6) Başlık satırı DOSYANIN İLK SATIRI olmalıdır; üstüne rapor başlığı eklemeyin.</v>
+        <v>5) Gece sayısı tarihlerden hesaplanır, ayrı sütun gerekmez.</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>7) Sütun sırası önemsizdir, fazladan sütunlar yok sayılır.</v>
+        <v>6) Başlık satırı DOSYANIN İLK SATIRI olmalıdır; üstüne rapor başlığı eklemeyin.</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>8) "Oda İndirimi" yalnız oda gelirinden düşer; temizlik ücretini etkilemez.</v>
+        <v>7) Sütun sırası önemsizdir, fazladan sütunlar yok sayılır.</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v xml:space="preserve">   "Telefon" ve "Not" isteğe bağlıdır.</v>
+        <v>8) "Oda İndirimi" yalnız oda gelirinden düşer; temizlik ücretini etkilemez.</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v/>
+        <v xml:space="preserve">   "Telefon" ve "Not" isteğe bağlıdır.</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
         <v>Durum değerleri: CONFIRMED, CHECKED_IN, CHECKED_OUT, CANCELLED</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:A19"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:A20"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>